<commit_message>
Auto-push ARPES website updates
</commit_message>
<xml_diff>
--- a/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
+++ b/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R73e2248413e54ea9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re962e202c68444f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="R426b96eaaf3b49a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R6395b15d23b74cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R65ff88b2340e4eea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="Rf9dc133597924927"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -946,6 +946,35 @@
         <x:v>本文件</x:v>
       </x:c>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="10" t="str">
+        <x:v>A022</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>魔方按草图改为左侧大透明六面体、右侧 Chat platform；周期表按草图改为左侧大周期表、右侧 Module/材料索引</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
+        <x:v>魔方/周期表界面</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G23" s="10" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="H23" s="10" t="str">
+        <x:v>继续按实际使用反馈细调空间比例和模块命名</x:v>
+      </x:c>
+      <x:c r="I23" s="10" t="str">
+        <x:v>用户 2026-06-25 两张手绘草图</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -980,7 +1009,7 @@
         <x:v>总建议数</x:v>
       </x:c>
       <x:c r="B2" s="10" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C2" s="10" t="str">
         <x:v>从本轮和前序讨论整理</x:v>
@@ -994,7 +1023,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B3" s="10" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>状态为 Done</x:v>
@@ -1163,13 +1192,27 @@
         <x:v>v0.9</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>current</x:v>
+        <x:v>be9470c</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
         <x:v>简洁主界面、注销、Word 报告、版本和销项清单</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="10" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>按手绘草图重排魔方和周期表工作台</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add report export format choices
</commit_message>
<xml_diff>
--- a/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
+++ b/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R6395b15d23b74cdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R65ff88b2340e4eea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="Rf9dc133597924927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R2bf1f9ba8e3f46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1f47965aa71c45c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="R43638d7b4dbc432c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -975,6 +975,35 @@
         <x:v>用户 2026-06-25 两张手绘草图</x:v>
       </x:c>
     </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="10" t="str">
+        <x:v>A023</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>生成调研报告时可选择 PDF、Word、Excel、Markdown 等格式</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>报告导出</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="H24" s="10" t="str">
+        <x:v>后续可接服务器端原生 PDF/Docx 生成</x:v>
+      </x:c>
+      <x:c r="I24" s="10" t="str">
+        <x:v>用户要求报告格式可选</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1009,7 +1038,7 @@
         <x:v>总建议数</x:v>
       </x:c>
       <x:c r="B2" s="10" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C2" s="10" t="str">
         <x:v>从本轮和前序讨论整理</x:v>
@@ -1023,7 +1052,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B3" s="10" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>状态为 Done</x:v>

</xml_diff>

<commit_message>
Add module roundtable to periodic view
</commit_message>
<xml_diff>
--- a/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
+++ b/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R63ecf766e9504f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R694d21c8693b4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="R07f22dc3a2f24a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R0e55239db5f0412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R4c4a7c58e4c44404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="R4d1db22d20d442f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1033,6 +1033,35 @@
         <x:v>用户要求修复看到的 bug</x:v>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="10" t="str">
+        <x:v>A025</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>周期表界面按草图改为左侧 periodic table，右侧圆桌上围绕 Module，而不是元素</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="str">
+        <x:v>周期表/模块导航</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str">
+        <x:v>v1.3</x:v>
+      </x:c>
+      <x:c r="H26" s="10" t="str">
+        <x:v>继续根据实际讨论调整圆桌模块名称和跳转目标</x:v>
+      </x:c>
+      <x:c r="I26" s="10" t="str">
+        <x:v>用户 2026-06-25 圆桌草图澄清</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1067,7 +1096,7 @@
         <x:v>总建议数</x:v>
       </x:c>
       <x:c r="B2" s="10" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="10" t="str">
         <x:v>从本轮和前序讨论整理</x:v>
@@ -1081,7 +1110,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B3" s="10" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>状态为 Done</x:v>
@@ -1292,13 +1321,27 @@
         <x:v>v1.2</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>current</x:v>
+        <x:v>c2ceb57</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
         <x:v>顶部工具栏和报告导出入口可用性修复</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="10" t="str">
+        <x:v>v1.3</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>周期表右侧 Module 圆桌导航</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Show full periodic table
</commit_message>
<xml_diff>
--- a/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
+++ b/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R0e55239db5f0412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R4c4a7c58e4c44404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="R4d1db22d20d442f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="Reb1c7948b6ef4795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R6e12c82a98e74cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="R313645b3a3114e2a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1062,6 +1062,35 @@
         <x:v>用户 2026-06-25 圆桌草图澄清</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="10" t="str">
+        <x:v>A026</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="str">
+        <x:v>元素周期表需要完整显示全部 118 个元素，有数据的高亮、暂无文献数据的置灰</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="str">
+        <x:v>周期表</x:v>
+      </x:c>
+      <x:c r="E27" s="10" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F27" s="10" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G27" s="10" t="str">
+        <x:v>v1.4</x:v>
+      </x:c>
+      <x:c r="H27" s="10" t="str">
+        <x:v>后续导入新文献后自动把对应元素从灰色变为可探索</x:v>
+      </x:c>
+      <x:c r="I27" s="10" t="str">
+        <x:v>用户要求元素周期表都显示出来</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1096,7 +1125,7 @@
         <x:v>总建议数</x:v>
       </x:c>
       <x:c r="B2" s="10" t="n">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C2" s="10" t="str">
         <x:v>从本轮和前序讨论整理</x:v>
@@ -1110,7 +1139,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B3" s="10" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>状态为 Done</x:v>
@@ -1335,13 +1364,27 @@
         <x:v>v1.3</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>current</x:v>
+        <x:v>0a9f372</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
         <x:v>周期表右侧 Module 圆桌导航</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="10" t="str">
+        <x:v>v1.4</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>完整 118 元素周期表显示</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Refine ARPES menu and chat report flow
</commit_message>
<xml_diff>
--- a/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
+++ b/outputs/arpes_action_checklist/arpes_discussion_action_items.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R57ad6ce6ee4d426f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7f0b5fd2e4d44106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="Rba6017edb7de4eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Checklist" sheetId="1" r:id="R087d1672e374440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rd44e07bd6d9d4773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Versions" sheetId="3" r:id="Rd4eff80fe99c4006"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -160,58 +160,12 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="67000"/>
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="73000"/>
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="81000"/>
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="94000"/>
-                <a:lumMod val="102000"/>
-                <a:satMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:shade val="100000"/>
-                <a:lumMod val="100000"/>
-                <a:satMod val="110000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="78000"/>
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="dk1"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="accent1"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -1120,6 +1074,35 @@
         <x:v>OpenAlex + arXiv + Crossref</x:v>
       </x:c>
     </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="10" t="str">
+        <x:v>A028</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>周期表做成单独界面，删除左侧电子书目录占位；Chat platform 负责问答、表格和报告导出；顶部菜单参考基金委风格</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
+        <x:v>主界面/Chat/report</x:v>
+      </x:c>
+      <x:c r="E29" s="10" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F29" s="10" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G29" s="10" t="str">
+        <x:v>v1.6</x:v>
+      </x:c>
+      <x:c r="H29" s="10" t="str">
+        <x:v>外部 AI 如豆包需后端代理和密钥，不能直接放 GitHub Pages 前端</x:v>
+      </x:c>
+      <x:c r="I29" s="10" t="str">
+        <x:v>用户 2026-06-26 参考图</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1154,7 +1137,7 @@
         <x:v>总建议数</x:v>
       </x:c>
       <x:c r="B2" s="10" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C2" s="10" t="str">
         <x:v>从本轮和前序讨论整理</x:v>
@@ -1168,7 +1151,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B3" s="10" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>状态为 Done</x:v>
@@ -1421,13 +1404,27 @@
         <x:v>v1.5</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>current</x:v>
+        <x:v>babb467</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
         <x:v>免费 ARPES API 元数据导入器</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="10" t="str">
+        <x:v>v1.6</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>current</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>顶部菜单、独立周期表界面和 Chat platform 报告导出</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>